<commit_message>
Owner Operational Performance rebuild, Owner PDF brief, sidebar icons, dashboard trends and (i) links
- O-09 Operational Performance: dashboard from the model (Group/A1/A2), anomaly heat map, entity charts
- Dashboard cards: prominent trend chip, hero colour follows risk (red = High risk only), (i) links to KPI Reference
- Heat map grid sized to its risk levels (was fixed at 4 columns and broke with 3)
- KPI Reference: scan_ui reads dashboard and heat blocks; graph source rules for O-03/O-09
- MANIFEST04: Owner brief rebuilt as a 2-page portrait PDF with IBM Plex Sans subset; report.js cache-buster
- MANIFEST05: sidebar SVG icons, white active tab with blue text
- tools/check_dash_master.js: 122 O-03/O-09 numbers checked against kpi_values.csv

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018hQtdmArgqT1EERTYJUBZb
</commit_message>
<xml_diff>
--- a/data/kpi-model/Group-KPI-Model.xlsx
+++ b/data/kpi-model/Group-KPI-Model.xlsx
@@ -680,7 +680,7 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>98.1%</t>
+          <t>95.5 % of plan</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>E-01,E-02,E-05,G-01,G-02,G-03,G-05,O-01,O-09,S-03,S-10,STATE GALLERY</t>
+          <t>O-01, O-09, E-01, E-02, E-05, G-01, G-02, G-03, G-05, S-03, S-10, STATE GALLERY</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
@@ -726,7 +726,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>83.4 %</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>E-02,G-05,O-01,STATE GALLERY</t>
+          <t>O-01, O-09, E-02, G-05, STATE GALLERY</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>78 %</t>
+          <t>84.1 %</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>E-02,G-05</t>
+          <t>O-09, E-02, G-05</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -944,7 +944,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>205 h</t>
+          <t>270 h</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>E-03,G-05,O-09</t>
+          <t>O-09, E-03, G-05</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>3.6 h</t>
+          <t>7.8 h</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>E-03,G-05,O-09</t>
+          <t>O-09, E-03, G-05</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>E-03,G-05,O-09</t>
+          <t>E-03, G-05</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>95.6 %</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>E-03,O-09</t>
+          <t>O-09, E-03</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>₹412 /t</t>
+          <t>2,934 ₹/t</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-11,G-03,G-05,O-09</t>
+          <t>O-09, E-02, E-11, G-03, G-05</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-11,G-03,O-09</t>
+          <t>E-02, E-11, G-03</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>E-02,O-09</t>
+          <t>E-02</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-07,G-05,G-07,O-05,O-09</t>
+          <t>O-05, E-02, E-07, G-05, G-07</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>0.82 tCO2e/t</t>
+          <t>427.7 kt CO2e</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-07,G-05,G-07,O-05,O-09</t>
+          <t>O-05, O-09, E-02, E-07, G-05, G-07</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-07,G-05,G-07,O-05,O-09</t>
+          <t>O-05, E-02, E-07, G-05, G-07</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>E-01,E-04,O-09,S-10,S-12</t>
+          <t>E-01, E-04, S-10, S-12</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>E-01,G-01,O-01,O-09</t>
+          <t>O-01, E-01, G-01</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -2128,17 +2128,17 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>78.4 %</t>
+          <t>Not on a screen</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Different</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>6.1 ₹/t</t>
+          <t>174 ₹/t</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
@@ -4290,17 +4290,17 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>91.4 %</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>Same</t>
+          <t>Different</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>E-04,G-05,O-09</t>
+          <t>O-09, E-04, G-05</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
@@ -4336,15 +4336,19 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Not shown</t>
+          <t>96.8 %</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr">
         <is>
-          <t>Not shown</t>
-        </is>
-      </c>
-      <c r="H82" s="3" t="n"/>
+          <t>Different</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>O-09</t>
+        </is>
+      </c>
       <c r="I82" s="3" t="inlineStr">
         <is>
           <t>Synthetic inputs added for this model</t>
@@ -4512,17 +4516,17 @@
       </c>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>Not on a screen</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>Different</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I86" s="3" t="inlineStr">
@@ -4558,17 +4562,17 @@
       </c>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Not on a screen</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>Different</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H87" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I87" s="3" t="inlineStr">
@@ -7190,7 +7194,7 @@
       </c>
       <c r="H144" s="3" t="inlineStr">
         <is>
-          <t>E-01,E-04,O-01,O-02,O-09,S-10,S-12,STATE GALLERY</t>
+          <t>O-01, O-02, E-01, E-04, S-10, S-12, STATE GALLERY</t>
         </is>
       </c>
       <c r="I144" s="3" t="inlineStr">
@@ -7420,7 +7424,7 @@
       </c>
       <c r="H149" s="3" t="inlineStr">
         <is>
-          <t>G-05,G-10,O-09</t>
+          <t>G-05, G-10</t>
         </is>
       </c>
       <c r="I149" s="3" t="inlineStr">
@@ -7456,17 +7460,17 @@
       </c>
       <c r="F150" s="3" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>Not on a screen</t>
         </is>
       </c>
       <c r="G150" s="5" t="inlineStr">
         <is>
-          <t>Different</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H150" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I150" s="3" t="inlineStr">
@@ -7625,12 +7629,12 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>98.1%</t>
+          <t>98.1%; 95.5 % of plan (O-09)</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>E-01,E-02,E-05,G-01,G-02,G-03,G-05,O-01,O-09,S-03,S-10,STATE GALLERY</t>
+          <t>O-01, O-09, E-01, E-02, E-05, G-01, G-02, G-03, G-05, S-03, S-10, STATE GALLERY</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
@@ -7691,12 +7695,12 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>86%</t>
+          <t>86%; 83.4 % (O-09)</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>E-02,G-05,O-01,STATE GALLERY</t>
+          <t>O-01, O-09, E-02, G-05, STATE GALLERY</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
@@ -7819,12 +7823,12 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>78 %</t>
+          <t>78 %; 84.1 % (O-09)</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>E-02,G-05</t>
+          <t>O-09, E-02, G-05</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
@@ -8009,12 +8013,12 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>205 h</t>
+          <t>205 h; 270 h (O-09)</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>E-03,G-05,O-09</t>
+          <t>O-09, E-03, G-05</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
@@ -8075,12 +8079,12 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>3.6 h</t>
+          <t>3.6 h; 7.8 h (O-09)</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>E-03,G-05,O-09</t>
+          <t>O-09, E-03, G-05</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
@@ -8146,7 +8150,7 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>E-03,G-05,O-09</t>
+          <t>E-03, G-05</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr">
@@ -8273,12 +8277,12 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>93%</t>
+          <t>93%; 95.6 % (O-09)</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>E-03,O-09</t>
+          <t>O-09, E-03</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
@@ -8339,12 +8343,12 @@
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>₹412 /t</t>
+          <t>₹412 /t; 2,934 ₹/t (O-09)</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-11,G-03,G-05,O-09</t>
+          <t>O-09, E-02, E-11, G-03, G-05</t>
         </is>
       </c>
       <c r="N13" s="3" t="inlineStr">
@@ -8410,7 +8414,7 @@
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-11,G-03,O-09</t>
+          <t>E-02, E-11, G-03</t>
         </is>
       </c>
       <c r="N14" s="3" t="inlineStr">
@@ -8476,7 +8480,7 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>E-02,O-09</t>
+          <t>E-02</t>
         </is>
       </c>
       <c r="N15" s="3" t="inlineStr">
@@ -8542,7 +8546,7 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-07,G-05,G-07,O-05,O-09</t>
+          <t>O-05, E-02, E-07, G-05, G-07</t>
         </is>
       </c>
       <c r="N16" s="3" t="inlineStr">
@@ -8603,12 +8607,12 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>0.82 tCO2e/t</t>
+          <t>0.82 tCO2e/t; 427.7 kt CO2e (O-09)</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-07,G-05,G-07,O-05,O-09</t>
+          <t>O-05, O-09, E-02, E-07, G-05, G-07</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr">
@@ -8674,7 +8678,7 @@
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>E-02,E-07,G-05,G-07,O-05,O-09</t>
+          <t>O-05, E-02, E-07, G-05, G-07</t>
         </is>
       </c>
       <c r="N18" s="3" t="inlineStr">
@@ -8864,7 +8868,7 @@
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>E-01,E-04,O-09,S-10,S-12</t>
+          <t>E-01, E-04, S-10, S-12</t>
         </is>
       </c>
       <c r="N21" s="3" t="inlineStr">
@@ -9652,7 +9656,7 @@
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>E-01,G-01,O-01,O-09</t>
+          <t>O-01, E-01, G-01</t>
         </is>
       </c>
       <c r="N33" s="3" t="inlineStr">
@@ -9718,7 +9722,7 @@
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N34" s="3" t="inlineStr">
@@ -9911,7 +9915,7 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>6.1 ₹/t</t>
+          <t>6.1 ₹/t; 174 ₹/t (O-09)</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr">
@@ -12815,12 +12819,12 @@
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t>91%</t>
+          <t>91%; 91.4 % (O-09)</t>
         </is>
       </c>
       <c r="M81" s="3" t="inlineStr">
         <is>
-          <t>E-04,G-05,O-09</t>
+          <t>O-09, E-04, G-05</t>
         </is>
       </c>
       <c r="N81" s="3" t="inlineStr">
@@ -12881,10 +12885,14 @@
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>Not shown</t>
-        </is>
-      </c>
-      <c r="M82" s="3" t="n"/>
+          <t>Not shown; 96.8 % (O-09)</t>
+        </is>
+      </c>
+      <c r="M82" s="3" t="inlineStr">
+        <is>
+          <t>O-09</t>
+        </is>
+      </c>
       <c r="N82" s="3" t="inlineStr">
         <is>
           <t>qty_ordered_t, qty_received_t</t>
@@ -13142,7 +13150,7 @@
       </c>
       <c r="M86" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N86" s="3" t="inlineStr">
@@ -13208,7 +13216,7 @@
       </c>
       <c r="M87" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N87" s="3" t="inlineStr">
@@ -16970,7 +16978,7 @@
       </c>
       <c r="M144" s="3" t="inlineStr">
         <is>
-          <t>E-01,E-04,O-01,O-02,O-09,S-10,S-12,STATE GALLERY</t>
+          <t>O-01, O-02, E-01, E-04, S-10, S-12, STATE GALLERY</t>
         </is>
       </c>
       <c r="N144" s="3" t="inlineStr">
@@ -17300,7 +17308,7 @@
       </c>
       <c r="M149" s="3" t="inlineStr">
         <is>
-          <t>G-05,G-10,O-09</t>
+          <t>G-05, G-10</t>
         </is>
       </c>
       <c r="N149" s="3" t="inlineStr">
@@ -17366,7 +17374,7 @@
       </c>
       <c r="M150" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N150" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Operational Performance: speedometer gauges, alert bar, heat map in the middle, charts at the bottom
- Gauge option on dashboard hero cards (all six templates): 240° dial, zones from the model target, needle, target marker; red only for High risk
- O-09: removed the secondary cards (A1/A2 production, MTTR, supplier OTD and fill rate, emissions, OEE, PM compliance, capacity); kept the three gauges and power cost
- Alert bar computed from the model inputs (A1 shortfall 30.3 kt, Group 29.4 kt) with a KPI strip; replaces the banner
- Charts moved to a second dashboard block under the heat map; tools read every dash block
- Workbooks and KPI Reference listings re-synced

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018hQtdmArgqT1EERTYJUBZb
</commit_message>
<xml_diff>
--- a/data/kpi-model/Group-KPI-Model.xlsx
+++ b/data/kpi-model/Group-KPI-Model.xlsx
@@ -736,7 +736,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>O-01, O-09, E-02, G-05, STATE GALLERY</t>
+          <t>O-01, E-02, G-05, STATE GALLERY</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>O-09, E-02, G-05</t>
+          <t>E-02, G-05</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>O-09, E-03, G-05</t>
+          <t>E-03, G-05</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>O-09, E-03</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>O-05, O-09, E-02, E-07, G-05, G-07</t>
+          <t>O-05, E-02, E-07, G-05, G-07</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="H81" s="3" t="inlineStr">
         <is>
-          <t>O-09, E-04, G-05</t>
+          <t>E-04, G-05</t>
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr">
@@ -4336,17 +4336,17 @@
       </c>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>96.8 %</t>
+          <t>Not on a screen</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr">
         <is>
-          <t>Different</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H82" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I82" s="3" t="inlineStr">
@@ -7695,12 +7695,12 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>86%; 83.4 % (O-09)</t>
+          <t>86%</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>O-01, O-09, E-02, G-05, STATE GALLERY</t>
+          <t>O-01, E-02, G-05, STATE GALLERY</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
@@ -7823,12 +7823,12 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>78 %; 84.1 % (O-09)</t>
+          <t>78 %</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>O-09, E-02, G-05</t>
+          <t>E-02, G-05</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
@@ -8079,12 +8079,12 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>3.6 h; 7.8 h (O-09)</t>
+          <t>3.6 h</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>O-09, E-03, G-05</t>
+          <t>E-03, G-05</t>
         </is>
       </c>
       <c r="N9" s="3" t="inlineStr">
@@ -8277,12 +8277,12 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>93%; 95.6 % (O-09)</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>O-09, E-03</t>
+          <t>E-03</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr">
@@ -8607,12 +8607,12 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>0.82 tCO2e/t; 427.7 kt CO2e (O-09)</t>
+          <t>0.82 tCO2e/t</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>O-05, O-09, E-02, E-07, G-05, G-07</t>
+          <t>O-05, E-02, E-07, G-05, G-07</t>
         </is>
       </c>
       <c r="N17" s="3" t="inlineStr">
@@ -12819,12 +12819,12 @@
       </c>
       <c r="L81" s="3" t="inlineStr">
         <is>
-          <t>91%; 91.4 % (O-09)</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="M81" s="3" t="inlineStr">
         <is>
-          <t>O-09, E-04, G-05</t>
+          <t>E-04, G-05</t>
         </is>
       </c>
       <c r="N81" s="3" t="inlineStr">
@@ -12885,12 +12885,12 @@
       </c>
       <c r="L82" s="3" t="inlineStr">
         <is>
-          <t>Not shown; 96.8 % (O-09)</t>
+          <t>Not shown</t>
         </is>
       </c>
       <c r="M82" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N82" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Operational Performance: remove the Power cost per tonne card
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018hQtdmArgqT1EERTYJUBZb
</commit_message>
<xml_diff>
--- a/data/kpi-model/Group-KPI-Model.xlsx
+++ b/data/kpi-model/Group-KPI-Model.xlsx
@@ -2266,17 +2266,17 @@
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>174 ₹/t</t>
+          <t>Not on a screen</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Different</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
@@ -9915,12 +9915,12 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>6.1 ₹/t; 174 ₹/t (O-09)</t>
+          <t>6.1 ₹/t</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t>O-09</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N37" s="3" t="inlineStr">

</xml_diff>